<commit_message>
Add orders from Orders_import, orders screen; fix empty stock row in SQL script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hp1yELqH2ftvHdxUjfdiCq
</commit_message>
<xml_diff>
--- a/chudo_obuv/Excel_3НФ.xlsx
+++ b/chudo_obuv/Excel_3НФ.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="products" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sizes" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stock" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="orders" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="order_items" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,6 +472,652 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>size_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2190</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2790</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>8565</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>22</v>
+      </c>
+      <c r="D8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7795</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7757</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>12340</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" t="n">
+        <v>17</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7130</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8765</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>11</v>
+      </c>
+      <c r="D13" t="n">
+        <v>17</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>25</v>
+      </c>
+      <c r="D14" t="n">
+        <v>28</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>9567</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>29</v>
+      </c>
+      <c r="D15" t="n">
+        <v>28</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>21500</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>24</v>
+      </c>
+      <c r="D16" t="n">
+        <v>17</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>7890</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D17" t="n">
+        <v>18</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>24569</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>6</v>
+      </c>
+      <c r="C18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" t="n">
+        <v>24</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>14567</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" t="n">
+        <v>31</v>
+      </c>
+      <c r="D19" t="n">
+        <v>28</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>15670</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4290</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2190</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" t="n">
+        <v>12</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="n">
+        <v>28</v>
+      </c>
+      <c r="D23" t="n">
+        <v>29</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>25625</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="n">
+        <v>24</v>
+      </c>
+      <c r="D24" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7890</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="n">
+        <v>23</v>
+      </c>
+      <c r="D25" t="n">
+        <v>26</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="n">
+        <v>6550</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>9</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2490</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>9</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3190</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>10</v>
+      </c>
+      <c r="C28" t="n">
+        <v>18</v>
+      </c>
+      <c r="D28" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>7550</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" t="n">
+        <v>15</v>
+      </c>
+      <c r="D29" t="n">
+        <v>16</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7130</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>10</v>
+      </c>
+      <c r="C30" t="n">
+        <v>16</v>
+      </c>
+      <c r="D30" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>12340</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="n">
+        <v>21</v>
+      </c>
+      <c r="D31" t="n">
+        <v>20</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>8765</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3019,7 +3667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4150,9 +4798,165 @@
         <v>30</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>order_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make user passwords empty so login works by login only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hp1yELqH2ftvHdxUjfdiCq
</commit_message>
<xml_diff>
--- a/chudo_obuv/Excel_3НФ.xlsx
+++ b/chudo_obuv/Excel_3НФ.xlsx
@@ -1188,11 +1188,7 @@
           <t>isivanov</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>1</v>
       </c>
@@ -1221,11 +1217,7 @@
           <t>papetrov</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>2</v>
       </c>
@@ -1254,11 +1246,7 @@
           <t>asidorova</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>3</v>
       </c>
@@ -1287,11 +1275,7 @@
           <t>ekuznetsova</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>2</v>
       </c>
@@ -1320,11 +1304,7 @@
           <t>dsmirnov</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>3</v>
       </c>
@@ -1353,11 +1333,7 @@
           <t>apopov</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>1</v>
       </c>
@@ -1386,11 +1362,7 @@
           <t>ovasileva</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>3</v>
       </c>
@@ -1419,11 +1391,7 @@
           <t>psokolov</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>2</v>
       </c>
@@ -1452,11 +1420,7 @@
           <t>tmikhailova</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>3</v>
       </c>
@@ -1485,11 +1449,7 @@
           <t>nnovikova</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>2</v>
       </c>
@@ -1518,11 +1478,7 @@
           <t>afedorov</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>1</v>
       </c>
@@ -1551,11 +1507,7 @@
           <t>smorozov</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>3</v>
       </c>
@@ -1584,11 +1536,7 @@
           <t>jvolkova</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>2</v>
       </c>
@@ -1617,11 +1565,7 @@
           <t>aalekseev</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>3</v>
       </c>
@@ -1650,11 +1594,7 @@
           <t>ilebedeva</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>3</v>
       </c>
@@ -1683,11 +1623,7 @@
           <t>negorov</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>2</v>
       </c>
@@ -1716,11 +1652,7 @@
           <t>epavlova</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
         <v>3</v>
       </c>
@@ -1749,11 +1681,7 @@
           <t>rkozlov</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
         <v>1</v>
       </c>
@@ -1782,11 +1710,7 @@
           <t>vstepanova</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>2</v>
       </c>
@@ -1815,11 +1739,7 @@
           <t>vnikolaev</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>123456</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
         <v>3</v>
       </c>

</xml_diff>